<commit_message>
data: cierre dia 2026-07-14_1724 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/Planes AASS/sincargosjunio.xlsx
+++ b/01_INPUTS/Planes AASS/sincargosjunio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Orbit\MATINAL_PENAFLOR\01_INPUTS\Planes AASS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBB2FE4B-BDB5-4365-B026-90A72B449568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{203729A0-8975-449E-AF47-9842DBE12E88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{8398F70B-36A8-4A9F-A50B-4A31C9FEDDC3}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="99">
   <si>
     <t>clientes</t>
   </si>
@@ -326,6 +326,12 @@
   </si>
   <si>
     <t>Smirnoff Flavours</t>
+  </si>
+  <si>
+    <t>CHEN ZHONGQING (SUPERMERCADO CRISOL)</t>
+  </si>
+  <si>
+    <t>AV PONTIN 534</t>
   </si>
 </sst>
 </file>
@@ -1274,7 +1280,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE5B0672-9B1D-4469-8532-36560150BC3A}">
-  <dimension ref="B1:I32"/>
+  <dimension ref="B1:I33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.42578125" style="1"/>
@@ -1906,6 +1912,23 @@
         <v>5</v>
       </c>
     </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B33" s="1">
+        <v>2083</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F33" s="4">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B32">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>

</xml_diff>